<commit_message>
CCDC excel file updates for the release 1.4.8
</commit_message>
<xml_diff>
--- a/InputFiles/ICDC/TC08_Canine_Study-PRECINCT01-Breed-GoldenRetriever.xlsx
+++ b/InputFiles/ICDC/TC08_Canine_Study-PRECINCT01-Breed-GoldenRetriever.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\epishinavv\git\Commons_Automation\InputFiles\ICDC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E60794D-1ADF-4DB3-9FF8-F0A535DAC78D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A34BD0B-06BD-44DD-9B8B-B306547F9701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{8362173B-D28C-47E7-8626-98E16101E601}"/>
   </bookViews>
@@ -159,7 +159,7 @@
     <t>MATCH (f:file)--&gt;(s:study)
 MATCH (s)&lt;--(c:case)&lt;--(diag:diagnosis)
 MATCH (c)&lt;--(demo:demographic)
-WHERE s.clinical_study_designation IN ['PRECINCT01'] and  demo.breed  IN ['Golden Retriever'] 
+WHERE s.clinical_study_designation IN ['PRECINCT01']  and demo.breed  IN ['Golden Retriever'] 
 WITH
         DISTINCT f, c, demo, diag, s,
         ['Bytes', 'KB', 'MB', 'GB', 'TB'] AS units,

</xml_diff>